<commit_message>
Update JSONs from Excel
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$415</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$416</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1318" uniqueCount="446">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1321" uniqueCount="447">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1360,6 +1360,9 @@
   </si>
   <si>
     <t>FERRETERIA JULIAN</t>
+  </si>
+  <si>
+    <t>FERRETERIA LUCKA</t>
   </si>
 </sst>
 </file>
@@ -1715,7 +1718,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D439"/>
+  <dimension ref="A1:D440"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6877,38 +6880,38 @@
     </row>
     <row r="369" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A369" s="6">
-        <v>61001</v>
-      </c>
-      <c r="B369" t="s">
-        <v>403</v>
+        <v>60305</v>
+      </c>
+      <c r="B369" s="18" t="s">
+        <v>446</v>
       </c>
       <c r="C369" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D369" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="370" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A370" s="6">
-        <v>61004</v>
+        <v>61001</v>
       </c>
       <c r="B370" t="s">
-        <v>293</v>
+        <v>403</v>
       </c>
       <c r="C370" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D370" s="15" t="s">
-        <v>5</v>
+      <c r="D370" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="371" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A371" s="6">
-        <v>61007</v>
+        <v>61004</v>
       </c>
       <c r="B371" t="s">
-        <v>415</v>
+        <v>293</v>
       </c>
       <c r="C371" s="1" t="s">
         <v>4</v>
@@ -6919,24 +6922,24 @@
     </row>
     <row r="372" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A372" s="6">
-        <v>61009</v>
+        <v>61007</v>
       </c>
       <c r="B372" t="s">
-        <v>294</v>
+        <v>415</v>
       </c>
       <c r="C372" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D372" s="12" t="s">
-        <v>8</v>
+      <c r="D372" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="373" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A373" s="6">
-        <v>61012</v>
+        <v>61009</v>
       </c>
       <c r="B373" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C373" s="1" t="s">
         <v>4</v>
@@ -6947,10 +6950,10 @@
     </row>
     <row r="374" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A374" s="6">
-        <v>61018</v>
+        <v>61012</v>
       </c>
       <c r="B374" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C374" s="1" t="s">
         <v>4</v>
@@ -6961,10 +6964,10 @@
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>61102</v>
+        <v>61018</v>
       </c>
       <c r="B375" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
@@ -6975,52 +6978,52 @@
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>61205</v>
+        <v>61102</v>
       </c>
       <c r="B376" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D376" s="15" t="s">
-        <v>5</v>
+      <c r="D376" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>70100</v>
+        <v>61205</v>
       </c>
       <c r="B377" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D377" s="12" t="s">
-        <v>8</v>
+      <c r="D377" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>70101</v>
+        <v>70100</v>
       </c>
       <c r="B378" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D378" s="15" t="s">
-        <v>5</v>
+      <c r="D378" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>70102</v>
+        <v>70101</v>
       </c>
       <c r="B379" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
@@ -7031,94 +7034,94 @@
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>70103</v>
+        <v>70102</v>
       </c>
       <c r="B380" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D380" s="12" t="s">
-        <v>8</v>
+      <c r="D380" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>70106</v>
+        <v>70103</v>
       </c>
       <c r="B381" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D381" s="15" t="s">
-        <v>5</v>
+      <c r="D381" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>70107</v>
+        <v>70106</v>
       </c>
       <c r="B382" t="s">
-        <v>419</v>
+        <v>303</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D382" s="15" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>70109</v>
+        <v>70107</v>
       </c>
       <c r="B383" t="s">
-        <v>304</v>
+        <v>419</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D383" s="12" t="s">
+      <c r="D383" s="15" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>70113</v>
+        <v>70109</v>
       </c>
       <c r="B384" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D384" s="15" t="s">
-        <v>5</v>
+      <c r="D384" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>70114</v>
+        <v>70113</v>
       </c>
       <c r="B385" t="s">
-        <v>325</v>
+        <v>305</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D385" s="9" t="s">
-        <v>9</v>
+      <c r="D385" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>70115</v>
+        <v>70114</v>
       </c>
       <c r="B386" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
@@ -7129,38 +7132,38 @@
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>70116</v>
+        <v>70115</v>
       </c>
       <c r="B387" t="s">
-        <v>420</v>
+        <v>331</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D387" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>70638</v>
+        <v>70116</v>
       </c>
       <c r="B388" t="s">
-        <v>306</v>
+        <v>420</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D388" s="12" t="s">
+      <c r="D388" s="9" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>70639</v>
+        <v>70638</v>
       </c>
       <c r="B389" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
@@ -7171,10 +7174,10 @@
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>70640</v>
+        <v>70639</v>
       </c>
       <c r="B390" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
@@ -7185,10 +7188,10 @@
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>70642</v>
+        <v>70640</v>
       </c>
       <c r="B391" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
@@ -7199,10 +7202,10 @@
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>90504</v>
+        <v>70642</v>
       </c>
       <c r="B392" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
@@ -7213,10 +7216,10 @@
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>90509</v>
+        <v>90504</v>
       </c>
       <c r="B393" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
@@ -7227,52 +7230,52 @@
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>90602</v>
+        <v>90509</v>
       </c>
       <c r="B394" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D394" s="15" t="s">
-        <v>5</v>
+      <c r="D394" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
-        <v>90621</v>
+        <v>90602</v>
       </c>
       <c r="B395" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C395" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D395" s="12" t="s">
-        <v>8</v>
+      <c r="D395" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6">
-        <v>90622</v>
+        <v>90621</v>
       </c>
       <c r="B396" t="s">
-        <v>333</v>
+        <v>313</v>
       </c>
       <c r="C396" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D396" s="9" t="s">
-        <v>5</v>
+      <c r="D396" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="397" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A397" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B397" s="8" t="s">
-        <v>342</v>
+        <v>90622</v>
+      </c>
+      <c r="B397" t="s">
+        <v>333</v>
       </c>
       <c r="C397" s="1" t="s">
         <v>4</v>
@@ -7283,24 +7286,24 @@
     </row>
     <row r="398" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6">
-        <v>90658</v>
-      </c>
-      <c r="B398" t="s">
-        <v>314</v>
+        <v>90631</v>
+      </c>
+      <c r="B398" s="8" t="s">
+        <v>342</v>
       </c>
       <c r="C398" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D398" s="12" t="s">
-        <v>8</v>
+      <c r="D398" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="399" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A399" s="6">
-        <v>90660</v>
+        <v>90658</v>
       </c>
       <c r="B399" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>4</v>
@@ -7311,10 +7314,10 @@
     </row>
     <row r="400" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A400" s="6">
-        <v>90668</v>
+        <v>90660</v>
       </c>
       <c r="B400" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C400" s="1" t="s">
         <v>4</v>
@@ -7325,10 +7328,10 @@
     </row>
     <row r="401" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A401" s="6">
-        <v>90671</v>
+        <v>90668</v>
       </c>
       <c r="B401" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C401" s="1" t="s">
         <v>4</v>
@@ -7339,10 +7342,10 @@
     </row>
     <row r="402" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A402" s="6">
-        <v>90679</v>
+        <v>90671</v>
       </c>
       <c r="B402" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C402" s="1" t="s">
         <v>4</v>
@@ -7353,10 +7356,10 @@
     </row>
     <row r="403" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A403" s="6">
-        <v>90683</v>
+        <v>90679</v>
       </c>
       <c r="B403" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C403" s="1" t="s">
         <v>4</v>
@@ -7367,10 +7370,10 @@
     </row>
     <row r="404" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A404" s="6">
-        <v>90705</v>
+        <v>90683</v>
       </c>
       <c r="B404" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C404" s="1" t="s">
         <v>4</v>
@@ -7381,10 +7384,10 @@
     </row>
     <row r="405" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A405" s="6">
-        <v>90706</v>
+        <v>90705</v>
       </c>
       <c r="B405" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C405" s="1" t="s">
         <v>4</v>
@@ -7395,10 +7398,10 @@
     </row>
     <row r="406" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A406" s="6">
-        <v>90708</v>
+        <v>90706</v>
       </c>
       <c r="B406" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C406" s="1" t="s">
         <v>4</v>
@@ -7409,10 +7412,10 @@
     </row>
     <row r="407" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A407" s="6">
-        <v>90709</v>
+        <v>90708</v>
       </c>
       <c r="B407" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C407" s="1" t="s">
         <v>4</v>
@@ -7423,38 +7426,38 @@
     </row>
     <row r="408" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A408" s="6">
-        <v>90713</v>
+        <v>90709</v>
       </c>
       <c r="B408" t="s">
-        <v>402</v>
+        <v>323</v>
       </c>
       <c r="C408" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D408" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="409" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A409" s="6">
-        <v>1218</v>
+        <v>90713</v>
       </c>
       <c r="B409" t="s">
-        <v>382</v>
+        <v>402</v>
       </c>
       <c r="C409" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D409" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="410" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A410" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B410" s="8" t="s">
-        <v>383</v>
+        <v>1218</v>
+      </c>
+      <c r="B410" t="s">
+        <v>382</v>
       </c>
       <c r="C410" s="1" t="s">
         <v>4</v>
@@ -7465,10 +7468,10 @@
     </row>
     <row r="411" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A411" s="6">
-        <v>5625</v>
+        <v>1959</v>
       </c>
       <c r="B411" s="8" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C411" s="1" t="s">
         <v>4</v>
@@ -7479,10 +7482,10 @@
     </row>
     <row r="412" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A412" s="6">
-        <v>1817</v>
+        <v>5625</v>
       </c>
       <c r="B412" s="8" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="C412" s="1" t="s">
         <v>4</v>
@@ -7493,10 +7496,10 @@
     </row>
     <row r="413" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A413" s="6">
-        <v>5737</v>
+        <v>1817</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C413" s="1" t="s">
         <v>4</v>
@@ -7507,68 +7510,68 @@
     </row>
     <row r="414" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A414" s="6">
-        <v>60295</v>
+        <v>5737</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C414" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D414" s="9" t="s">
-        <v>9</v>
+      <c r="D414" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="415" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A415" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B415" s="8" t="s">
+        <v>385</v>
+      </c>
+      <c r="C415" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D415" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="416" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A416" s="6">
         <v>1045</v>
       </c>
-      <c r="B415" s="8" t="s">
+      <c r="B416" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C415" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D415" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="416" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A416">
-        <v>1043</v>
-      </c>
-      <c r="B416" t="s">
-        <v>422</v>
-      </c>
-      <c r="C416" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D416" t="s">
-        <v>8</v>
+      <c r="C416" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D416" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="417" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A417">
+        <v>1043</v>
+      </c>
+      <c r="B417" t="s">
+        <v>422</v>
+      </c>
+      <c r="C417" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D417" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="418" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A418">
         <v>20340</v>
       </c>
-      <c r="B417" t="s">
+      <c r="B418" t="s">
         <v>423</v>
       </c>
-      <c r="C417" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D417" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="418" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A418">
-        <v>40146</v>
-      </c>
-      <c r="B418" t="s">
-        <v>424</v>
-      </c>
-      <c r="C418" s="14" t="s">
+      <c r="C418" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D418" t="s">
@@ -7577,24 +7580,24 @@
     </row>
     <row r="419" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A419">
-        <v>60260</v>
+        <v>40146</v>
       </c>
       <c r="B419" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C419" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D419" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="420" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A420">
-        <v>1017</v>
+        <v>60260</v>
       </c>
       <c r="B420" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C420" s="14" t="s">
         <v>4</v>
@@ -7605,10 +7608,10 @@
     </row>
     <row r="421" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A421">
-        <v>60300</v>
+        <v>1017</v>
       </c>
       <c r="B421" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C421" s="14" t="s">
         <v>4</v>
@@ -7619,66 +7622,66 @@
     </row>
     <row r="422" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A422">
-        <v>20191</v>
+        <v>60300</v>
       </c>
       <c r="B422" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C422" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D422" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="423" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A423">
-        <v>20399</v>
+        <v>20191</v>
       </c>
       <c r="B423" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C423" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D423" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="424" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A424">
-        <v>60240</v>
+        <v>20399</v>
       </c>
       <c r="B424" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C424" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D424" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="425" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A425">
-        <v>60244</v>
+        <v>60240</v>
       </c>
       <c r="B425" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C425" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D425" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="426" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A426">
-        <v>60248</v>
+        <v>60244</v>
       </c>
       <c r="B426" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C426" s="14" t="s">
         <v>4</v>
@@ -7689,24 +7692,24 @@
     </row>
     <row r="427" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A427">
-        <v>60288</v>
+        <v>60248</v>
       </c>
       <c r="B427" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C427" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D427" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="428" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A428">
-        <v>90714</v>
+        <v>60288</v>
       </c>
       <c r="B428" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C428" s="14" t="s">
         <v>4</v>
@@ -7717,10 +7720,10 @@
     </row>
     <row r="429" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A429">
-        <v>1014</v>
+        <v>90714</v>
       </c>
       <c r="B429" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C429" s="14" t="s">
         <v>4</v>
@@ -7731,38 +7734,38 @@
     </row>
     <row r="430" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A430">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="B430" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C430" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D430" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="431" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A431">
-        <v>60301</v>
+        <v>1016</v>
       </c>
       <c r="B431" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C431" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D431" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="432" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A432">
-        <v>1041</v>
+        <v>60301</v>
       </c>
       <c r="B432" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C432" s="14" t="s">
         <v>4</v>
@@ -7773,10 +7776,10 @@
     </row>
     <row r="433" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A433">
-        <v>971</v>
+        <v>1041</v>
       </c>
       <c r="B433" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C433" s="14" t="s">
         <v>4</v>
@@ -7787,38 +7790,38 @@
     </row>
     <row r="434" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A434">
-        <v>50610</v>
+        <v>971</v>
       </c>
       <c r="B434" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C434" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D434" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="435" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>943</v>
+        <v>50610</v>
       </c>
       <c r="B435" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C435" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D435" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="436" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A436">
-        <v>20306</v>
+        <v>943</v>
       </c>
       <c r="B436" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C436" s="14" t="s">
         <v>4</v>
@@ -7829,24 +7832,24 @@
     </row>
     <row r="437" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>90630</v>
+        <v>20306</v>
       </c>
       <c r="B437" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C437" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D437" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="438" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>1047</v>
+        <v>90630</v>
       </c>
       <c r="B438" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C438" s="14" t="s">
         <v>4</v>
@@ -7857,20 +7860,34 @@
     </row>
     <row r="439" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A439">
+        <v>1047</v>
+      </c>
+      <c r="B439" t="s">
+        <v>444</v>
+      </c>
+      <c r="C439" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D439" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="440" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A440">
         <v>20398</v>
       </c>
-      <c r="B439" t="s">
+      <c r="B440" t="s">
         <v>445</v>
       </c>
-      <c r="C439" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D439" t="s">
+      <c r="C440" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D440" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D415"/>
+  <autoFilter ref="A1:D416"/>
   <sortState ref="A2:D374">
     <sortCondition ref="A277"/>
   </sortState>

</xml_diff>

<commit_message>
update estado de cuentas
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$420</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -1380,7 +1380,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -6159,7 +6159,7 @@
         <v>4</v>
       </c>
       <c r="D316" s="10" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="317" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Actualizar los precios sin recargar cuando cambia el catalogo, Promociones: solo con cliente elegido y precio de lista completo en el panel
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$445</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$447</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="454">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1378,12 +1378,18 @@
   </si>
   <si>
     <t>FERRETERIA CLAUDIO</t>
+  </si>
+  <si>
+    <t>FERRETERIA RyV</t>
+  </si>
+  <si>
+    <t>FERRETERIA A y J</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -1733,7 +1739,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D445"/>
+  <dimension ref="A1:D447"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6979,80 +6985,80 @@
     </row>
     <row r="375" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A375" s="6">
-        <v>61001</v>
-      </c>
-      <c r="B375" t="s">
-        <v>394</v>
+        <v>60306</v>
+      </c>
+      <c r="B375" s="18" t="s">
+        <v>453</v>
       </c>
       <c r="C375" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D375" s="12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="376" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A376" s="6">
-        <v>61004</v>
-      </c>
-      <c r="B376" t="s">
-        <v>287</v>
+        <v>60308</v>
+      </c>
+      <c r="B376" s="18" t="s">
+        <v>452</v>
       </c>
       <c r="C376" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D376" s="15" t="s">
-        <v>5</v>
+      <c r="D376" s="12" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="377" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A377" s="6">
-        <v>61007</v>
+        <v>61001</v>
       </c>
       <c r="B377" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="C377" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D377" s="15" t="s">
-        <v>5</v>
+      <c r="D377" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="378" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A378" s="6">
-        <v>61009</v>
+        <v>61004</v>
       </c>
       <c r="B378" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C378" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D378" s="12" t="s">
-        <v>8</v>
+      <c r="D378" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="379" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A379" s="6">
-        <v>61012</v>
+        <v>61007</v>
       </c>
       <c r="B379" t="s">
-        <v>289</v>
+        <v>405</v>
       </c>
       <c r="C379" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D379" s="12" t="s">
-        <v>8</v>
+      <c r="D379" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="380" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A380" s="6">
-        <v>61018</v>
+        <v>61009</v>
       </c>
       <c r="B380" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C380" s="1" t="s">
         <v>4</v>
@@ -7063,10 +7069,10 @@
     </row>
     <row r="381" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A381" s="6">
-        <v>61102</v>
+        <v>61012</v>
       </c>
       <c r="B381" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C381" s="1" t="s">
         <v>4</v>
@@ -7077,24 +7083,24 @@
     </row>
     <row r="382" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A382" s="6">
-        <v>61205</v>
+        <v>61018</v>
       </c>
       <c r="B382" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C382" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D382" s="15" t="s">
-        <v>5</v>
+      <c r="D382" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="383" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A383" s="6">
-        <v>70100</v>
+        <v>61102</v>
       </c>
       <c r="B383" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C383" s="1" t="s">
         <v>4</v>
@@ -7105,10 +7111,10 @@
     </row>
     <row r="384" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A384" s="6">
-        <v>70101</v>
+        <v>61205</v>
       </c>
       <c r="B384" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C384" s="1" t="s">
         <v>4</v>
@@ -7119,38 +7125,38 @@
     </row>
     <row r="385" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A385" s="6">
-        <v>70102</v>
+        <v>70100</v>
       </c>
       <c r="B385" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C385" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D385" s="15" t="s">
-        <v>5</v>
+      <c r="D385" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="386" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A386" s="6">
-        <v>70103</v>
+        <v>70101</v>
       </c>
       <c r="B386" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C386" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D386" s="12" t="s">
-        <v>8</v>
+      <c r="D386" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="387" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A387" s="6">
-        <v>70106</v>
+        <v>70102</v>
       </c>
       <c r="B387" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C387" s="1" t="s">
         <v>4</v>
@@ -7161,122 +7167,122 @@
     </row>
     <row r="388" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A388" s="6">
-        <v>70107</v>
+        <v>70103</v>
       </c>
       <c r="B388" t="s">
-        <v>409</v>
+        <v>296</v>
       </c>
       <c r="C388" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D388" s="15" t="s">
+      <c r="D388" s="12" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="389" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A389" s="6">
-        <v>70109</v>
+        <v>70106</v>
       </c>
       <c r="B389" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C389" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D389" s="12" t="s">
-        <v>8</v>
+      <c r="D389" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="390" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A390" s="6">
-        <v>70113</v>
+        <v>70107</v>
       </c>
       <c r="B390" t="s">
-        <v>299</v>
+        <v>409</v>
       </c>
       <c r="C390" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D390" s="15" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="391" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6">
-        <v>70114</v>
+        <v>70109</v>
       </c>
       <c r="B391" t="s">
-        <v>319</v>
+        <v>298</v>
       </c>
       <c r="C391" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D391" s="9" t="s">
-        <v>9</v>
+      <c r="D391" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="392" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6">
-        <v>70115</v>
+        <v>70113</v>
       </c>
       <c r="B392" t="s">
-        <v>325</v>
+        <v>299</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D392" s="9" t="s">
-        <v>9</v>
+      <c r="D392" s="15" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="393" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6">
-        <v>70116</v>
+        <v>70114</v>
       </c>
       <c r="B393" t="s">
-        <v>410</v>
+        <v>319</v>
       </c>
       <c r="C393" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D393" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="394" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6">
-        <v>70638</v>
+        <v>70115</v>
       </c>
       <c r="B394" t="s">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="C394" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D394" s="12" t="s">
-        <v>8</v>
+      <c r="D394" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="395" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6">
-        <v>70639</v>
+        <v>70116</v>
       </c>
       <c r="B395" t="s">
-        <v>301</v>
+        <v>410</v>
       </c>
       <c r="C395" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D395" s="12" t="s">
+      <c r="D395" s="9" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="396" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6">
-        <v>70640</v>
+        <v>70638</v>
       </c>
       <c r="B396" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C396" s="1" t="s">
         <v>4</v>
@@ -7287,10 +7293,10 @@
     </row>
     <row r="397" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A397" s="6">
-        <v>70642</v>
+        <v>70639</v>
       </c>
       <c r="B397" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C397" s="1" t="s">
         <v>4</v>
@@ -7301,10 +7307,10 @@
     </row>
     <row r="398" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6">
-        <v>90504</v>
+        <v>70640</v>
       </c>
       <c r="B398" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C398" s="1" t="s">
         <v>4</v>
@@ -7315,10 +7321,10 @@
     </row>
     <row r="399" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A399" s="6">
-        <v>90509</v>
+        <v>70642</v>
       </c>
       <c r="B399" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>4</v>
@@ -7329,24 +7335,24 @@
     </row>
     <row r="400" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A400" s="6">
-        <v>90602</v>
+        <v>90504</v>
       </c>
       <c r="B400" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C400" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D400" s="15" t="s">
-        <v>5</v>
+      <c r="D400" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="401" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A401" s="6">
-        <v>90621</v>
+        <v>90509</v>
       </c>
       <c r="B401" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C401" s="1" t="s">
         <v>4</v>
@@ -7357,66 +7363,66 @@
     </row>
     <row r="402" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A402" s="6">
-        <v>90622</v>
+        <v>90602</v>
       </c>
       <c r="B402" t="s">
-        <v>327</v>
+        <v>306</v>
       </c>
       <c r="C402" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D402" s="9" t="s">
+      <c r="D402" s="15" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="403" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A403" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B403" s="8" t="s">
-        <v>336</v>
+        <v>90621</v>
+      </c>
+      <c r="B403" t="s">
+        <v>307</v>
       </c>
       <c r="C403" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D403" s="9" t="s">
-        <v>5</v>
+      <c r="D403" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="404" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A404" s="6">
-        <v>90658</v>
+        <v>90622</v>
       </c>
       <c r="B404" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="C404" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D404" s="12" t="s">
-        <v>8</v>
+      <c r="D404" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="405" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A405" s="6">
-        <v>90660</v>
-      </c>
-      <c r="B405" t="s">
-        <v>309</v>
+        <v>90631</v>
+      </c>
+      <c r="B405" s="8" t="s">
+        <v>336</v>
       </c>
       <c r="C405" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D405" s="12" t="s">
-        <v>8</v>
+      <c r="D405" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="406" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A406" s="6">
-        <v>90668</v>
+        <v>90658</v>
       </c>
       <c r="B406" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C406" s="1" t="s">
         <v>4</v>
@@ -7427,10 +7433,10 @@
     </row>
     <row r="407" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A407" s="6">
-        <v>90671</v>
+        <v>90660</v>
       </c>
       <c r="B407" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C407" s="1" t="s">
         <v>4</v>
@@ -7441,10 +7447,10 @@
     </row>
     <row r="408" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A408" s="6">
-        <v>90679</v>
+        <v>90668</v>
       </c>
       <c r="B408" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C408" s="1" t="s">
         <v>4</v>
@@ -7455,10 +7461,10 @@
     </row>
     <row r="409" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A409" s="6">
-        <v>90683</v>
+        <v>90671</v>
       </c>
       <c r="B409" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C409" s="1" t="s">
         <v>4</v>
@@ -7469,10 +7475,10 @@
     </row>
     <row r="410" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A410" s="6">
-        <v>90705</v>
+        <v>90679</v>
       </c>
       <c r="B410" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C410" s="1" t="s">
         <v>4</v>
@@ -7483,10 +7489,10 @@
     </row>
     <row r="411" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A411" s="6">
-        <v>90706</v>
+        <v>90683</v>
       </c>
       <c r="B411" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C411" s="1" t="s">
         <v>4</v>
@@ -7497,10 +7503,10 @@
     </row>
     <row r="412" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A412" s="6">
-        <v>90708</v>
+        <v>90705</v>
       </c>
       <c r="B412" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C412" s="1" t="s">
         <v>4</v>
@@ -7511,10 +7517,10 @@
     </row>
     <row r="413" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A413" s="6">
-        <v>90709</v>
+        <v>90706</v>
       </c>
       <c r="B413" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C413" s="1" t="s">
         <v>4</v>
@@ -7525,24 +7531,24 @@
     </row>
     <row r="414" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A414" s="6">
-        <v>90713</v>
+        <v>90708</v>
       </c>
       <c r="B414" t="s">
-        <v>393</v>
+        <v>316</v>
       </c>
       <c r="C414" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D414" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="415" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A415" s="6">
-        <v>1218</v>
+        <v>90709</v>
       </c>
       <c r="B415" t="s">
-        <v>373</v>
+        <v>317</v>
       </c>
       <c r="C415" s="1" t="s">
         <v>4</v>
@@ -7553,24 +7559,24 @@
     </row>
     <row r="416" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A416" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B416" s="8" t="s">
-        <v>374</v>
+        <v>90713</v>
+      </c>
+      <c r="B416" t="s">
+        <v>393</v>
       </c>
       <c r="C416" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D416" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="417" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A417" s="6">
-        <v>5625</v>
-      </c>
-      <c r="B417" s="8" t="s">
-        <v>375</v>
+        <v>1218</v>
+      </c>
+      <c r="B417" t="s">
+        <v>373</v>
       </c>
       <c r="C417" s="1" t="s">
         <v>4</v>
@@ -7581,10 +7587,10 @@
     </row>
     <row r="418" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A418" s="6">
-        <v>1817</v>
+        <v>1959</v>
       </c>
       <c r="B418" s="8" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="C418" s="1" t="s">
         <v>4</v>
@@ -7595,10 +7601,10 @@
     </row>
     <row r="419" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A419" s="6">
-        <v>5737</v>
+        <v>5625</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="C419" s="1" t="s">
         <v>4</v>
@@ -7609,108 +7615,108 @@
     </row>
     <row r="420" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A420" s="6">
-        <v>60295</v>
+        <v>1817</v>
       </c>
       <c r="B420" s="8" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="C420" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D420" s="9" t="s">
-        <v>9</v>
+      <c r="D420" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="421" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A421" s="6">
+        <v>5737</v>
+      </c>
+      <c r="B421" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="C421" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D421" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="422" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A422" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B422" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="C422" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D422" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="423" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A423" s="6">
         <v>1045</v>
       </c>
-      <c r="B421" s="8" t="s">
+      <c r="B423" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="C421" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D421" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="422" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A422">
+      <c r="C423" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D423" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="424" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A424">
         <v>1043</v>
       </c>
-      <c r="B422" t="s">
+      <c r="B424" t="s">
         <v>412</v>
       </c>
-      <c r="C422" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D422" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="423" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A423">
+      <c r="C424" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D424" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="425" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A425">
         <v>20340</v>
       </c>
-      <c r="B423" t="s">
+      <c r="B425" t="s">
         <v>413</v>
       </c>
-      <c r="C423" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D423" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="424" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A424">
-        <v>40146</v>
-      </c>
-      <c r="B424" t="s">
-        <v>414</v>
-      </c>
-      <c r="C424" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D424" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="425" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A425">
-        <v>60260</v>
-      </c>
-      <c r="B425" t="s">
-        <v>415</v>
-      </c>
-      <c r="C425" s="14" t="s">
+      <c r="C425" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D425" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="426" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A426">
-        <v>1017</v>
+        <v>40146</v>
       </c>
       <c r="B426" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="C426" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D426" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="427" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A427">
-        <v>60300</v>
+        <v>60260</v>
       </c>
       <c r="B427" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C427" s="14" t="s">
         <v>4</v>
@@ -7721,24 +7727,24 @@
     </row>
     <row r="428" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A428">
-        <v>20191</v>
+        <v>1017</v>
       </c>
       <c r="B428" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C428" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D428" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="429" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A429">
-        <v>20399</v>
+        <v>60300</v>
       </c>
       <c r="B429" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C429" s="14" t="s">
         <v>4</v>
@@ -7749,10 +7755,10 @@
     </row>
     <row r="430" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A430">
-        <v>60240</v>
+        <v>20191</v>
       </c>
       <c r="B430" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C430" s="14" t="s">
         <v>4</v>
@@ -7763,10 +7769,10 @@
     </row>
     <row r="431" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A431">
-        <v>60244</v>
+        <v>20399</v>
       </c>
       <c r="B431" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C431" s="14" t="s">
         <v>4</v>
@@ -7777,52 +7783,52 @@
     </row>
     <row r="432" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A432">
-        <v>60248</v>
+        <v>60240</v>
       </c>
       <c r="B432" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C432" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D432" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="433" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A433">
-        <v>60288</v>
+        <v>60244</v>
       </c>
       <c r="B433" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C433" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D433" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="434" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A434">
-        <v>90714</v>
+        <v>60248</v>
       </c>
       <c r="B434" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C434" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D434" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="435" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>1014</v>
+        <v>60288</v>
       </c>
       <c r="B435" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C435" s="14" t="s">
         <v>4</v>
@@ -7833,24 +7839,24 @@
     </row>
     <row r="436" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A436">
-        <v>1016</v>
+        <v>90714</v>
       </c>
       <c r="B436" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C436" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D436" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="437" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>60301</v>
+        <v>1014</v>
       </c>
       <c r="B437" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C437" s="14" t="s">
         <v>4</v>
@@ -7861,24 +7867,24 @@
     </row>
     <row r="438" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>1041</v>
+        <v>1016</v>
       </c>
       <c r="B438" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C438" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D438" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="439" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A439">
-        <v>971</v>
+        <v>60301</v>
       </c>
       <c r="B439" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C439" s="14" t="s">
         <v>4</v>
@@ -7889,24 +7895,24 @@
     </row>
     <row r="440" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A440">
-        <v>50610</v>
+        <v>1041</v>
       </c>
       <c r="B440" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C440" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D440" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="441" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A441">
-        <v>943</v>
+        <v>971</v>
       </c>
       <c r="B441" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C441" s="14" t="s">
         <v>4</v>
@@ -7917,62 +7923,90 @@
     </row>
     <row r="442" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A442">
-        <v>20306</v>
+        <v>50610</v>
       </c>
       <c r="B442" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C442" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D442" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="443" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A443">
-        <v>90630</v>
+        <v>943</v>
       </c>
       <c r="B443" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C443" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D443" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="444" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A444">
-        <v>1047</v>
+        <v>20306</v>
       </c>
       <c r="B444" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C444" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D444" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="445" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A445">
+        <v>90630</v>
+      </c>
+      <c r="B445" t="s">
+        <v>433</v>
+      </c>
+      <c r="C445" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D445" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="446" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A446">
+        <v>1047</v>
+      </c>
+      <c r="B446" t="s">
+        <v>434</v>
+      </c>
+      <c r="C446" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D446" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="447" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A447">
         <v>20398</v>
       </c>
-      <c r="B445" t="s">
+      <c r="B447" t="s">
         <v>435</v>
       </c>
-      <c r="C445" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D445" t="s">
+      <c r="C447" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D447" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D445"/>
+  <autoFilter ref="A1:D447"/>
   <sortState ref="A2:D374">
     <sortCondition ref="A277"/>
   </sortState>

</xml_diff>

<commit_message>
Regenerar el indice de busqueda con los productos nuevos
</commit_message>
<xml_diff>
--- a/excel/CLIENTES_PERMISOS.xlsx
+++ b/excel/CLIENTES_PERMISOS.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$449</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja 1'!$A$1:$D$451</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1348" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1357" uniqueCount="459">
   <si>
     <t>CUENTA</t>
   </si>
@@ -1390,6 +1390,15 @@
   </si>
   <si>
     <t>DEPO P.BAJA</t>
+  </si>
+  <si>
+    <t>F. RAUCH ADRIAN</t>
+  </si>
+  <si>
+    <t>FERRETERIA ANIBAL</t>
+  </si>
+  <si>
+    <t>FERRETERIA VALVERDE</t>
   </si>
 </sst>
 </file>
@@ -1745,7 +1754,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D449"/>
+  <dimension ref="A1:D452"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6090,7 +6099,7 @@
         <v>4</v>
       </c>
       <c r="D310" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="311" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6580,7 +6589,7 @@
         <v>4</v>
       </c>
       <c r="D345" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="346" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7313,38 +7322,38 @@
     </row>
     <row r="398" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6">
-        <v>70638</v>
+        <v>70117</v>
       </c>
       <c r="B398" t="s">
-        <v>300</v>
+        <v>457</v>
       </c>
       <c r="C398" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D398" s="12" t="s">
-        <v>8</v>
+      <c r="D398" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="399" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A399" s="6">
-        <v>70639</v>
+        <v>70118</v>
       </c>
       <c r="B399" t="s">
-        <v>301</v>
+        <v>458</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D399" s="12" t="s">
-        <v>8</v>
+      <c r="D399" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="400" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A400" s="6">
-        <v>70640</v>
+        <v>70638</v>
       </c>
       <c r="B400" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C400" s="1" t="s">
         <v>4</v>
@@ -7355,10 +7364,10 @@
     </row>
     <row r="401" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A401" s="6">
-        <v>70642</v>
+        <v>70639</v>
       </c>
       <c r="B401" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C401" s="1" t="s">
         <v>4</v>
@@ -7369,10 +7378,10 @@
     </row>
     <row r="402" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A402" s="6">
-        <v>90504</v>
+        <v>70640</v>
       </c>
       <c r="B402" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C402" s="1" t="s">
         <v>4</v>
@@ -7383,10 +7392,10 @@
     </row>
     <row r="403" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A403" s="6">
-        <v>90509</v>
+        <v>70642</v>
       </c>
       <c r="B403" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C403" s="1" t="s">
         <v>4</v>
@@ -7397,94 +7406,94 @@
     </row>
     <row r="404" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A404" s="6">
-        <v>90602</v>
+        <v>90504</v>
       </c>
       <c r="B404" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C404" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D404" s="15" t="s">
-        <v>5</v>
+      <c r="D404" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="405" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A405" s="6">
-        <v>90621</v>
+        <v>90509</v>
       </c>
       <c r="B405" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C405" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D405" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="406" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A406" s="6">
-        <v>90622</v>
+        <v>90602</v>
       </c>
       <c r="B406" t="s">
-        <v>327</v>
+        <v>306</v>
       </c>
       <c r="C406" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D406" s="9" t="s">
+      <c r="D406" s="15" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="407" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A407" s="6">
-        <v>90631</v>
-      </c>
-      <c r="B407" s="8" t="s">
-        <v>336</v>
+        <v>90621</v>
+      </c>
+      <c r="B407" t="s">
+        <v>307</v>
       </c>
       <c r="C407" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D407" s="9" t="s">
+      <c r="D407" s="12" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="408" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A408" s="6">
-        <v>90658</v>
+        <v>90622</v>
       </c>
       <c r="B408" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="C408" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D408" s="12" t="s">
-        <v>8</v>
+      <c r="D408" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="409" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A409" s="6">
-        <v>90660</v>
-      </c>
-      <c r="B409" t="s">
-        <v>309</v>
+        <v>90631</v>
+      </c>
+      <c r="B409" s="8" t="s">
+        <v>336</v>
       </c>
       <c r="C409" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D409" s="12" t="s">
-        <v>8</v>
+      <c r="D409" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="410" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A410" s="6">
-        <v>90668</v>
+        <v>90658</v>
       </c>
       <c r="B410" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C410" s="1" t="s">
         <v>4</v>
@@ -7495,10 +7504,10 @@
     </row>
     <row r="411" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A411" s="6">
-        <v>90671</v>
+        <v>90660</v>
       </c>
       <c r="B411" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C411" s="1" t="s">
         <v>4</v>
@@ -7509,10 +7518,10 @@
     </row>
     <row r="412" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A412" s="6">
-        <v>90679</v>
+        <v>90668</v>
       </c>
       <c r="B412" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C412" s="1" t="s">
         <v>4</v>
@@ -7523,10 +7532,10 @@
     </row>
     <row r="413" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A413" s="6">
-        <v>90683</v>
+        <v>90671</v>
       </c>
       <c r="B413" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C413" s="1" t="s">
         <v>4</v>
@@ -7537,10 +7546,10 @@
     </row>
     <row r="414" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A414" s="6">
-        <v>90705</v>
+        <v>90679</v>
       </c>
       <c r="B414" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C414" s="1" t="s">
         <v>4</v>
@@ -7551,10 +7560,10 @@
     </row>
     <row r="415" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A415" s="6">
-        <v>90706</v>
+        <v>90683</v>
       </c>
       <c r="B415" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C415" s="1" t="s">
         <v>4</v>
@@ -7565,10 +7574,10 @@
     </row>
     <row r="416" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A416" s="6">
-        <v>90708</v>
+        <v>90705</v>
       </c>
       <c r="B416" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C416" s="1" t="s">
         <v>4</v>
@@ -7579,10 +7588,10 @@
     </row>
     <row r="417" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A417" s="6">
-        <v>90709</v>
+        <v>90706</v>
       </c>
       <c r="B417" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C417" s="1" t="s">
         <v>4</v>
@@ -7593,24 +7602,24 @@
     </row>
     <row r="418" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A418" s="6">
-        <v>90713</v>
+        <v>90708</v>
       </c>
       <c r="B418" t="s">
-        <v>393</v>
+        <v>316</v>
       </c>
       <c r="C418" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D418" s="12" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="419" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A419" s="6">
-        <v>1218</v>
+        <v>90709</v>
       </c>
       <c r="B419" t="s">
-        <v>373</v>
+        <v>317</v>
       </c>
       <c r="C419" s="1" t="s">
         <v>4</v>
@@ -7621,24 +7630,24 @@
     </row>
     <row r="420" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A420" s="6">
-        <v>1959</v>
-      </c>
-      <c r="B420" s="8" t="s">
-        <v>374</v>
+        <v>90713</v>
+      </c>
+      <c r="B420" t="s">
+        <v>393</v>
       </c>
       <c r="C420" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D420" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="421" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A421" s="6">
-        <v>5625</v>
-      </c>
-      <c r="B421" s="8" t="s">
-        <v>375</v>
+        <v>1218</v>
+      </c>
+      <c r="B421" t="s">
+        <v>373</v>
       </c>
       <c r="C421" s="1" t="s">
         <v>4</v>
@@ -7649,10 +7658,10 @@
     </row>
     <row r="422" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A422" s="6">
-        <v>1817</v>
+        <v>1959</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="C422" s="1" t="s">
         <v>4</v>
@@ -7663,10 +7672,10 @@
     </row>
     <row r="423" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A423" s="6">
-        <v>5737</v>
+        <v>5625</v>
       </c>
       <c r="B423" s="8" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="C423" s="1" t="s">
         <v>4</v>
@@ -7677,108 +7686,108 @@
     </row>
     <row r="424" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A424" s="6">
-        <v>60295</v>
+        <v>1817</v>
       </c>
       <c r="B424" s="8" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="C424" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D424" s="9" t="s">
-        <v>9</v>
+      <c r="D424" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="425" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A425" s="6">
+        <v>5737</v>
+      </c>
+      <c r="B425" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="C425" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D425" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="426" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A426" s="6">
+        <v>60295</v>
+      </c>
+      <c r="B426" s="8" t="s">
+        <v>376</v>
+      </c>
+      <c r="C426" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D426" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="427" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A427" s="6">
         <v>1045</v>
       </c>
-      <c r="B425" s="8" t="s">
+      <c r="B427" s="8" t="s">
         <v>377</v>
       </c>
-      <c r="C425" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D425" s="9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="426" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A426">
+      <c r="C427" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D427" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="428" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A428">
         <v>1043</v>
       </c>
-      <c r="B426" t="s">
+      <c r="B428" t="s">
         <v>412</v>
       </c>
-      <c r="C426" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D426" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="427" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A427">
+      <c r="C428" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D428" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="429" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A429">
         <v>20340</v>
       </c>
-      <c r="B427" t="s">
+      <c r="B429" t="s">
         <v>413</v>
       </c>
-      <c r="C427" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D427" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="428" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A428">
-        <v>40146</v>
-      </c>
-      <c r="B428" t="s">
-        <v>414</v>
-      </c>
-      <c r="C428" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D428" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="429" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A429">
-        <v>60260</v>
-      </c>
-      <c r="B429" t="s">
-        <v>415</v>
-      </c>
-      <c r="C429" s="14" t="s">
+      <c r="C429" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D429" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="430" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A430">
-        <v>1017</v>
+        <v>40146</v>
       </c>
       <c r="B430" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="C430" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D430" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="431" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A431">
-        <v>60300</v>
+        <v>60260</v>
       </c>
       <c r="B431" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C431" s="14" t="s">
         <v>4</v>
@@ -7789,24 +7798,24 @@
     </row>
     <row r="432" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A432">
-        <v>20191</v>
+        <v>1017</v>
       </c>
       <c r="B432" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C432" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D432" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="433" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A433">
-        <v>20399</v>
+        <v>60300</v>
       </c>
       <c r="B433" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C433" s="14" t="s">
         <v>4</v>
@@ -7817,10 +7826,10 @@
     </row>
     <row r="434" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A434">
-        <v>60240</v>
+        <v>20191</v>
       </c>
       <c r="B434" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C434" s="14" t="s">
         <v>4</v>
@@ -7831,10 +7840,10 @@
     </row>
     <row r="435" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>60244</v>
+        <v>20399</v>
       </c>
       <c r="B435" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C435" s="14" t="s">
         <v>4</v>
@@ -7845,80 +7854,80 @@
     </row>
     <row r="436" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A436">
-        <v>60248</v>
+        <v>60240</v>
       </c>
       <c r="B436" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C436" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D436" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="437" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>60288</v>
+        <v>60244</v>
       </c>
       <c r="B437" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C437" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D437" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="438" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>90714</v>
+        <v>60248</v>
       </c>
       <c r="B438" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C438" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D438" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="439" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A439">
-        <v>1014</v>
+        <v>60288</v>
       </c>
       <c r="B439" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C439" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D439" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="440" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A440">
-        <v>1016</v>
+        <v>90714</v>
       </c>
       <c r="B440" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C440" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D440" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="441" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A441">
-        <v>60301</v>
+        <v>1014</v>
       </c>
       <c r="B441" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C441" s="14" t="s">
         <v>4</v>
@@ -7929,24 +7938,24 @@
     </row>
     <row r="442" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A442">
-        <v>1041</v>
+        <v>1016</v>
       </c>
       <c r="B442" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C442" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D442" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="443" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A443">
-        <v>971</v>
+        <v>60301</v>
       </c>
       <c r="B443" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C443" s="14" t="s">
         <v>4</v>
@@ -7957,24 +7966,24 @@
     </row>
     <row r="444" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A444">
-        <v>50610</v>
+        <v>1041</v>
       </c>
       <c r="B444" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C444" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D444" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="445" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A445">
-        <v>943</v>
+        <v>971</v>
       </c>
       <c r="B445" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C445" s="14" t="s">
         <v>4</v>
@@ -7985,62 +7994,104 @@
     </row>
     <row r="446" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A446">
-        <v>20306</v>
+        <v>50610</v>
       </c>
       <c r="B446" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C446" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D446" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="447" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A447">
-        <v>90630</v>
+        <v>943</v>
       </c>
       <c r="B447" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C447" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D447" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="448" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A448">
-        <v>1047</v>
+        <v>20306</v>
       </c>
       <c r="B448" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C448" s="14" t="s">
         <v>4</v>
       </c>
       <c r="D448" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="449" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A449">
+        <v>90630</v>
+      </c>
+      <c r="B449" t="s">
+        <v>433</v>
+      </c>
+      <c r="C449" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D449" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="450" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A450">
+        <v>1047</v>
+      </c>
+      <c r="B450" t="s">
+        <v>434</v>
+      </c>
+      <c r="C450" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D450" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="451" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A451">
         <v>20398</v>
       </c>
-      <c r="B449" t="s">
+      <c r="B451" t="s">
         <v>435</v>
       </c>
-      <c r="C449" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D449" t="s">
-        <v>8</v>
+      <c r="C451" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D451" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="452" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A452">
+        <v>50226</v>
+      </c>
+      <c r="B452" t="s">
+        <v>456</v>
+      </c>
+      <c r="C452" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D452" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D449"/>
+  <autoFilter ref="A1:D451"/>
   <sortState ref="A2:D374">
     <sortCondition ref="A277"/>
   </sortState>

</xml_diff>